<commit_message>
chore: push all recent changes to v1
</commit_message>
<xml_diff>
--- a/data_dict/member eligibility data dictitonary.xlsx
+++ b/data_dict/member eligibility data dictitonary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\AI\Phase II\healthcare_sql_generator\data_dict\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\AI\phase III - new\AI-Automation-III\data_dict\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE875C4-BA7C-45AA-9D1E-1BD86153E0FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B8C80FC-1B9F-4583-9B72-B018A0B1CD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{AD71633D-6DE9-4011-8424-5511CF23BF40}"/>
   </bookViews>
@@ -20,17 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -218,15 +207,6 @@
     <t>CoverageType</t>
   </si>
   <si>
-    <t>Type of benefit coverage</t>
-  </si>
-  <si>
-    <t>Medical</t>
-  </si>
-  <si>
-    <t>Medical, Dental, Vision, etc.</t>
-  </si>
-  <si>
     <t>CoverageStatus</t>
   </si>
   <si>
@@ -444,6 +424,19 @@
   </si>
   <si>
     <t>Indicates disability status</t>
+  </si>
+  <si>
+    <t>E, ECH, FAM</t>
+  </si>
+  <si>
+    <t>Coverage types_x000D_
+E : Employee only_x000D_
+F : Family_x000D_
+ECH : Employee + Children_x000D_
+ES : Employee + Spouse</t>
+  </si>
+  <si>
+    <t>Employee</t>
   </si>
 </sst>
 </file>
@@ -1190,49 +1183,49 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>59</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>60</v>
+        <v>134</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>61</v>
+        <v>133</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>62</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>12</v>
@@ -1241,13 +1234,13 @@
     </row>
     <row r="21" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>12</v>
@@ -1256,13 +1249,13 @@
     </row>
     <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>12</v>
@@ -1271,10 +1264,10 @@
     </row>
     <row r="23" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>33</v>
@@ -1286,10 +1279,10 @@
     </row>
     <row r="24" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>36</v>
@@ -1303,10 +1296,10 @@
     </row>
     <row r="25" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C25" s="4">
         <v>78701</v>
@@ -1320,30 +1313,30 @@
     </row>
     <row r="26" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>12</v>
@@ -1352,13 +1345,13 @@
     </row>
     <row r="28" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>12</v>
@@ -1367,27 +1360,27 @@
     </row>
     <row r="29" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C30" s="7">
         <v>45292</v>
@@ -1401,10 +1394,10 @@
     </row>
     <row r="31" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C31" s="5">
         <v>45657</v>
@@ -1418,13 +1411,13 @@
     </row>
     <row r="32" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>12</v>
@@ -1433,10 +1426,10 @@
     </row>
     <row r="33" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C33" s="4">
         <v>2109876543</v>
@@ -1445,15 +1438,15 @@
         <v>40</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C34" s="3">
         <v>300001</v>
@@ -1462,143 +1455,143 @@
         <v>7</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>123</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -1645,6 +1638,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010071CFE3CF7D33084FBE4C747B2C789FA3" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c28ef89bbeb6f449904cc4e79f5ef4ff">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="b0abcbf2-9bac-4e52-8a7c-5f8273d59732" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="642b821bee0c618b7c24cdb1870f8762" ns3:_="">
     <xsd:import namespace="b0abcbf2-9bac-4e52-8a7c-5f8273d59732"/>
@@ -1794,15 +1796,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1812,6 +1805,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{335AA437-C9A2-4990-8068-5A97F0EED3AE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5593D0AD-3186-4D9C-A651-35384A265607}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1825,14 +1826,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{335AA437-C9A2-4990-8068-5A97F0EED3AE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>